<commit_message>
Start preparing data files to correlate between them
</commit_message>
<xml_diff>
--- a/test_data/icpms_test/Picking_Test.xlsx
+++ b/test_data/icpms_test/Picking_Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Daven/Projects/Sparrow/Labs/Sparrow-CU-TRaIL/test_data/icpms_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F77B719-5B9D-8D4B-9E7B-4C9A58F0F252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6FF897-C1B0-F04F-B3D7-2A43A61CF6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="760" windowWidth="25880" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1486,8 +1486,8 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="str">
-        <f t="shared" ref="G7:G29" si="12">CONCATENATE(E7,"_",F7)</f>
-        <v>TestAp_1</v>
+        <f>CONCATENATE(E7,"_",TEXT(F7, "00"))</f>
+        <v>TestAp_01</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>82</v>
@@ -1544,46 +1544,46 @@
         <v>27931</v>
       </c>
       <c r="AA7" s="9">
-        <f t="shared" ref="AA7:AA29" si="13">(1/1.249)*AI7+(1-(1/1.249))*AJ7</f>
+        <f t="shared" ref="AA7:AA29" si="12">(1/1.249)*AI7+(1-(1/1.249))*AJ7</f>
         <v>0.7625501749135235</v>
       </c>
       <c r="AB7" s="9">
-        <f t="shared" ref="AB7:AB29" si="14">(1/1.249)*AK7+(1-(1/1.249))*AL7</f>
+        <f t="shared" ref="AB7:AB29" si="13">(1/1.249)*AK7+(1-(1/1.249))*AL7</f>
         <v>0.8528703850265964</v>
       </c>
       <c r="AD7" s="15" t="s">
         <v>39</v>
       </c>
       <c r="AE7" s="7">
-        <f t="shared" ref="AE7:AE27" si="15">(2.31*AG7+2*AH7)/(AH7*AG7)</f>
+        <f t="shared" ref="AE7:AE27" si="14">(2.31*AG7+2*AH7)/(AH7*AG7)</f>
         <v>4.8108127158965848E-2</v>
       </c>
       <c r="AF7" s="7">
-        <f t="shared" ref="AF7:AF27" si="16">(4*AG7+4+AH7)/(AG7*2*AH7)</f>
+        <f t="shared" ref="AF7:AF27" si="15">(4*AG7+4+AH7)/(AG7*2*AH7)</f>
         <v>3.4497793635661175E-2</v>
       </c>
       <c r="AG7" s="7">
-        <f t="shared" ref="AG7:AG27" si="17">(R7+T7)/2</f>
+        <f t="shared" ref="AG7:AG27" si="16">(R7+T7)/2</f>
         <v>167.77</v>
       </c>
       <c r="AH7" s="7">
-        <f t="shared" ref="AH7:AH27" si="18">(S7+U7)/4</f>
+        <f t="shared" ref="AH7:AH27" si="17">(S7+U7)/4</f>
         <v>63.835000000000001</v>
       </c>
       <c r="AI7" s="7">
-        <f t="shared" ref="AI7:AI27" si="19">1+(-5.13)*AE7+(6.79)*AE7^2</f>
+        <f t="shared" ref="AI7:AI27" si="18">1+(-5.13)*AE7+(6.79)*AE7^2</f>
         <v>0.76892002866697173</v>
       </c>
       <c r="AJ7" s="7">
-        <f t="shared" ref="AJ7:AJ27" si="20">1+(-5.9)*AE7+8.99*AE7^2</f>
+        <f t="shared" ref="AJ7:AJ27" si="19">1+(-5.9)*AE7+8.99*AE7^2</f>
         <v>0.73696843293180314</v>
       </c>
       <c r="AK7" s="7">
-        <f t="shared" ref="AK7:AK27" si="21">1+(-4.31)*AF7+4.92*AF7^2</f>
+        <f t="shared" ref="AK7:AK27" si="20">1+(-4.31)*AF7+4.92*AF7^2</f>
         <v>0.85716979043768537</v>
       </c>
       <c r="AL7" s="7">
-        <f t="shared" ref="AL7:AL27" si="22">1+(-5)*AF7+6.8*AF7^2</f>
+        <f t="shared" ref="AL7:AL27" si="21">1+(-5)*AF7+6.8*AF7^2</f>
         <v>0.83560369662864897</v>
       </c>
     </row>
@@ -1608,8 +1608,8 @@
         <v>2</v>
       </c>
       <c r="G8" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_2</v>
+        <f t="shared" ref="G8:G37" si="22">CONCATENATE(E8,"_",TEXT(F8, "00"))</f>
+        <v>TestAp_02</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>82</v>
@@ -1666,46 +1666,46 @@
         <v>27931</v>
       </c>
       <c r="AA8" s="9">
+        <f t="shared" si="12"/>
+        <v>0.77507947163167612</v>
+      </c>
+      <c r="AB8" s="9">
         <f t="shared" si="13"/>
-        <v>0.77507947163167612</v>
-      </c>
-      <c r="AB8" s="9">
-        <f t="shared" si="14"/>
         <v>0.8631274690997276</v>
       </c>
       <c r="AD8" s="15" t="s">
         <v>50</v>
       </c>
       <c r="AE8" s="7">
+        <f t="shared" si="14"/>
+        <v>4.538889222622583E-2</v>
+      </c>
+      <c r="AF8" s="7">
         <f t="shared" si="15"/>
-        <v>4.538889222622583E-2</v>
-      </c>
-      <c r="AF8" s="7">
+        <v>3.1993317722898852E-2</v>
+      </c>
+      <c r="AG8" s="7">
         <f t="shared" si="16"/>
-        <v>3.1993317722898852E-2</v>
-      </c>
-      <c r="AG8" s="7">
+        <v>164.67000000000002</v>
+      </c>
+      <c r="AH8" s="7">
         <f t="shared" si="17"/>
-        <v>164.67000000000002</v>
-      </c>
-      <c r="AH8" s="7">
+        <v>69.487499999999997</v>
+      </c>
+      <c r="AI8" s="7">
         <f t="shared" si="18"/>
-        <v>69.487499999999997</v>
-      </c>
-      <c r="AI8" s="7">
+        <v>0.78114341181924907</v>
+      </c>
+      <c r="AJ8" s="7">
         <f t="shared" si="19"/>
-        <v>0.78114341181924907</v>
-      </c>
-      <c r="AJ8" s="7">
+        <v>0.75072629818760783</v>
+      </c>
+      <c r="AK8" s="7">
         <f t="shared" si="20"/>
-        <v>0.75072629818760783</v>
-      </c>
-      <c r="AK8" s="7">
+        <v>0.86714477671858425</v>
+      </c>
+      <c r="AL8" s="7">
         <f t="shared" si="21"/>
-        <v>0.86714477671858425</v>
-      </c>
-      <c r="AL8" s="7">
-        <f t="shared" si="22"/>
         <v>0.84699370356215054</v>
       </c>
     </row>
@@ -1730,8 +1730,8 @@
         <v>3</v>
       </c>
       <c r="G9" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_3</v>
+        <f t="shared" si="22"/>
+        <v>TestAp_03</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>82</v>
@@ -1788,46 +1788,46 @@
         <v>27931</v>
       </c>
       <c r="AA9" s="9">
+        <f t="shared" si="12"/>
+        <v>0.78371827385864301</v>
+      </c>
+      <c r="AB9" s="9">
         <f t="shared" si="13"/>
-        <v>0.78371827385864301</v>
-      </c>
-      <c r="AB9" s="9">
-        <f t="shared" si="14"/>
         <v>0.8642899313368253</v>
       </c>
       <c r="AD9" s="15" t="s">
         <v>96</v>
       </c>
       <c r="AE9" s="7">
+        <f t="shared" si="14"/>
+        <v>4.3527389265401423E-2</v>
+      </c>
+      <c r="AF9" s="7">
         <f t="shared" si="15"/>
-        <v>4.3527389265401423E-2</v>
-      </c>
-      <c r="AF9" s="7">
+        <v>3.1710498042024214E-2</v>
+      </c>
+      <c r="AG9" s="7">
         <f t="shared" si="16"/>
-        <v>3.1710498042024214E-2</v>
-      </c>
-      <c r="AG9" s="7">
+        <v>201.24</v>
+      </c>
+      <c r="AH9" s="7">
         <f t="shared" si="17"/>
-        <v>201.24</v>
-      </c>
-      <c r="AH9" s="7">
+        <v>68.772500000000008</v>
+      </c>
+      <c r="AI9" s="7">
         <f t="shared" si="18"/>
-        <v>68.772500000000008</v>
-      </c>
-      <c r="AI9" s="7">
+        <v>0.78956905532290822</v>
+      </c>
+      <c r="AJ9" s="7">
         <f t="shared" si="19"/>
-        <v>0.78956905532290822</v>
-      </c>
-      <c r="AJ9" s="7">
+        <v>0.76022115954432501</v>
+      </c>
+      <c r="AK9" s="7">
         <f t="shared" si="20"/>
-        <v>0.76022115954432501</v>
-      </c>
-      <c r="AK9" s="7">
+        <v>0.86827508741435588</v>
+      </c>
+      <c r="AL9" s="7">
         <f t="shared" si="21"/>
-        <v>0.86827508741435588</v>
-      </c>
-      <c r="AL9" s="7">
-        <f t="shared" si="22"/>
         <v>0.84828528845517681</v>
       </c>
     </row>
@@ -1852,8 +1852,8 @@
         <v>4</v>
       </c>
       <c r="G10" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_4</v>
+        <f t="shared" si="22"/>
+        <v>TestAp_04</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>82</v>
@@ -1910,46 +1910,46 @@
         <v>27931</v>
       </c>
       <c r="AA10" s="9">
+        <f t="shared" si="12"/>
+        <v>0.66585244837043989</v>
+      </c>
+      <c r="AB10" s="9">
         <f t="shared" si="13"/>
-        <v>0.66585244837043989</v>
-      </c>
-      <c r="AB10" s="9">
-        <f t="shared" si="14"/>
         <v>0.79434370327453729</v>
       </c>
       <c r="AD10" s="15" t="s">
         <v>40</v>
       </c>
       <c r="AE10" s="7">
+        <f t="shared" si="14"/>
+        <v>6.9934964617649045E-2</v>
+      </c>
+      <c r="AF10" s="7">
         <f t="shared" si="15"/>
-        <v>6.9934964617649045E-2</v>
-      </c>
-      <c r="AF10" s="7">
+        <v>4.9111697732592205E-2</v>
+      </c>
+      <c r="AG10" s="7">
         <f t="shared" si="16"/>
-        <v>4.9111697732592205E-2</v>
-      </c>
-      <c r="AG10" s="7">
+        <v>103.84</v>
+      </c>
+      <c r="AH10" s="7">
         <f t="shared" si="17"/>
-        <v>103.84</v>
-      </c>
-      <c r="AH10" s="7">
+        <v>45.585000000000001</v>
+      </c>
+      <c r="AI10" s="7">
         <f t="shared" si="18"/>
-        <v>45.585000000000001</v>
-      </c>
-      <c r="AI10" s="7">
+        <v>0.67444283759598811</v>
+      </c>
+      <c r="AJ10" s="7">
         <f t="shared" si="19"/>
-        <v>0.67444283759598811</v>
-      </c>
-      <c r="AJ10" s="7">
+        <v>0.63135289324775634</v>
+      </c>
+      <c r="AK10" s="7">
         <f t="shared" si="20"/>
-        <v>0.63135289324775634</v>
-      </c>
-      <c r="AK10" s="7">
+        <v>0.80019542033508095</v>
+      </c>
+      <c r="AL10" s="7">
         <f t="shared" si="21"/>
-        <v>0.80019542033508095</v>
-      </c>
-      <c r="AL10" s="7">
-        <f t="shared" si="22"/>
         <v>0.77084283154544597</v>
       </c>
     </row>
@@ -1974,8 +1974,8 @@
         <v>5</v>
       </c>
       <c r="G11" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_5</v>
+        <f t="shared" si="22"/>
+        <v>TestAp_05</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>82</v>
@@ -2032,46 +2032,46 @@
         <v>27931</v>
       </c>
       <c r="AA11" s="9">
+        <f t="shared" si="12"/>
+        <v>0.84955136687159882</v>
+      </c>
+      <c r="AB11" s="9">
         <f t="shared" si="13"/>
-        <v>0.84955136687159882</v>
-      </c>
-      <c r="AB11" s="9">
-        <f t="shared" si="14"/>
         <v>0.9218973072509733</v>
       </c>
       <c r="AD11" s="15" t="s">
         <v>16</v>
       </c>
       <c r="AE11" s="7">
+        <f t="shared" si="14"/>
+        <v>2.9680377839805785E-2</v>
+      </c>
+      <c r="AF11" s="7">
         <f t="shared" si="15"/>
-        <v>2.9680377839805785E-2</v>
-      </c>
-      <c r="AF11" s="7">
+        <v>1.794413324859373E-2</v>
+      </c>
+      <c r="AG11" s="7">
         <f t="shared" si="16"/>
-        <v>1.794413324859373E-2</v>
-      </c>
-      <c r="AG11" s="7">
+        <v>156.96</v>
+      </c>
+      <c r="AH11" s="7">
         <f t="shared" si="17"/>
-        <v>156.96</v>
-      </c>
-      <c r="AH11" s="7">
+        <v>136.3775</v>
+      </c>
+      <c r="AI11" s="7">
         <f t="shared" si="18"/>
-        <v>136.3775</v>
-      </c>
-      <c r="AI11" s="7">
+        <v>0.85372114126876186</v>
+      </c>
+      <c r="AJ11" s="7">
         <f t="shared" si="19"/>
-        <v>0.85372114126876186</v>
-      </c>
-      <c r="AJ11" s="7">
+        <v>0.83280528495528139</v>
+      </c>
+      <c r="AK11" s="7">
         <f t="shared" si="20"/>
-        <v>0.83280528495528139</v>
-      </c>
-      <c r="AK11" s="7">
+        <v>0.924244985935334</v>
+      </c>
+      <c r="AL11" s="7">
         <f t="shared" si="21"/>
-        <v>0.924244985935334</v>
-      </c>
-      <c r="AL11" s="7">
-        <f t="shared" si="22"/>
         <v>0.91246887879972571</v>
       </c>
     </row>
@@ -2096,8 +2096,8 @@
         <v>6</v>
       </c>
       <c r="G12" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_6</v>
+        <f t="shared" si="22"/>
+        <v>TestAp_06</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>82</v>
@@ -2154,46 +2154,46 @@
         <v>27931</v>
       </c>
       <c r="AA12" s="9">
+        <f t="shared" si="12"/>
+        <v>0.62009648476517842</v>
+      </c>
+      <c r="AB12" s="9">
         <f t="shared" si="13"/>
-        <v>0.62009648476517842</v>
-      </c>
-      <c r="AB12" s="9">
-        <f t="shared" si="14"/>
         <v>0.77303373280373044</v>
       </c>
       <c r="AD12" s="15" t="s">
         <v>17</v>
       </c>
       <c r="AE12" s="7">
+        <f t="shared" si="14"/>
+        <v>8.0845937129300119E-2</v>
+      </c>
+      <c r="AF12" s="7">
         <f t="shared" si="15"/>
-        <v>8.0845937129300119E-2</v>
-      </c>
-      <c r="AF12" s="7">
+        <v>5.4577834618426253E-2</v>
+      </c>
+      <c r="AG12" s="7">
         <f t="shared" si="16"/>
-        <v>5.4577834618426253E-2</v>
-      </c>
-      <c r="AG12" s="7">
+        <v>76.8</v>
+      </c>
+      <c r="AH12" s="7">
         <f t="shared" si="17"/>
-        <v>76.8</v>
-      </c>
-      <c r="AH12" s="7">
+        <v>42.15</v>
+      </c>
+      <c r="AI12" s="7">
         <f t="shared" si="18"/>
-        <v>42.15</v>
-      </c>
-      <c r="AI12" s="7">
+        <v>0.62964022761332761</v>
+      </c>
+      <c r="AJ12" s="7">
         <f t="shared" si="19"/>
-        <v>0.62964022761332761</v>
-      </c>
-      <c r="AJ12" s="7">
+        <v>0.58176820023445885</v>
+      </c>
+      <c r="AK12" s="7">
         <f t="shared" si="20"/>
-        <v>0.58176820023445885</v>
-      </c>
-      <c r="AK12" s="7">
+        <v>0.77942493375023347</v>
+      </c>
+      <c r="AL12" s="7">
         <f t="shared" si="21"/>
-        <v>0.77942493375023347</v>
-      </c>
-      <c r="AL12" s="7">
-        <f t="shared" si="22"/>
         <v>0.74736625912299548</v>
       </c>
     </row>
@@ -2218,8 +2218,8 @@
         <v>7</v>
       </c>
       <c r="G13" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_7</v>
+        <f t="shared" si="22"/>
+        <v>TestAp_07</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>82</v>
@@ -2276,46 +2276,46 @@
         <v>27931</v>
       </c>
       <c r="AA13" s="9">
+        <f t="shared" si="12"/>
+        <v>0.58075299759262944</v>
+      </c>
+      <c r="AB13" s="9">
         <f t="shared" si="13"/>
-        <v>0.58075299759262944</v>
-      </c>
-      <c r="AB13" s="9">
-        <f t="shared" si="14"/>
         <v>0.75206879091305512</v>
       </c>
       <c r="AD13" s="15" t="s">
         <v>27</v>
       </c>
       <c r="AE13" s="7">
+        <f t="shared" si="14"/>
+        <v>9.0573869840029658E-2</v>
+      </c>
+      <c r="AF13" s="7">
         <f t="shared" si="15"/>
-        <v>9.0573869840029658E-2</v>
-      </c>
-      <c r="AF13" s="7">
+        <v>6.0036461620138031E-2</v>
+      </c>
+      <c r="AG13" s="7">
         <f t="shared" si="16"/>
-        <v>6.0036461620138031E-2</v>
-      </c>
-      <c r="AG13" s="7">
+        <v>64.2</v>
+      </c>
+      <c r="AH13" s="7">
         <f t="shared" si="17"/>
-        <v>64.2</v>
-      </c>
-      <c r="AH13" s="7">
+        <v>38.875</v>
+      </c>
+      <c r="AI13" s="7">
         <f t="shared" si="18"/>
-        <v>38.875</v>
-      </c>
-      <c r="AI13" s="7">
+        <v>0.59105866756670056</v>
+      </c>
+      <c r="AJ13" s="7">
         <f t="shared" si="19"/>
-        <v>0.59105866756670056</v>
-      </c>
-      <c r="AJ13" s="7">
+        <v>0.5393647647650347</v>
+      </c>
+      <c r="AK13" s="7">
         <f t="shared" si="20"/>
-        <v>0.5393647647650347</v>
-      </c>
-      <c r="AK13" s="7">
+        <v>0.75897638389862732</v>
+      </c>
+      <c r="AL13" s="7">
         <f t="shared" si="21"/>
-        <v>0.75897638389862732</v>
-      </c>
-      <c r="AL13" s="7">
-        <f t="shared" si="22"/>
         <v>0.72432745362160078</v>
       </c>
     </row>
@@ -2340,8 +2340,8 @@
         <v>8</v>
       </c>
       <c r="G14" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_8</v>
+        <f t="shared" si="22"/>
+        <v>TestAp_08</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>82</v>
@@ -2398,46 +2398,46 @@
         <v>27931</v>
       </c>
       <c r="AA14" s="9">
+        <f t="shared" si="12"/>
+        <v>0.59671359311517336</v>
+      </c>
+      <c r="AB14" s="9">
         <f t="shared" si="13"/>
-        <v>0.59671359311517336</v>
-      </c>
-      <c r="AB14" s="9">
-        <f t="shared" si="14"/>
         <v>0.72570314279312353</v>
       </c>
       <c r="AD14" s="15" t="s">
         <v>97</v>
       </c>
       <c r="AE14" s="7">
+        <f t="shared" si="14"/>
+        <v>8.6586598039484264E-2</v>
+      </c>
+      <c r="AF14" s="7">
         <f t="shared" si="15"/>
-        <v>8.6586598039484264E-2</v>
-      </c>
-      <c r="AF14" s="7">
+        <v>6.7021082876346977E-2</v>
+      </c>
+      <c r="AG14" s="7">
         <f t="shared" si="16"/>
-        <v>6.7021082876346977E-2</v>
-      </c>
-      <c r="AG14" s="7">
+        <v>147.05000000000001</v>
+      </c>
+      <c r="AH14" s="7">
         <f t="shared" si="17"/>
-        <v>147.05000000000001</v>
-      </c>
-      <c r="AH14" s="7">
+        <v>31.650000000000002</v>
+      </c>
+      <c r="AI14" s="7">
         <f t="shared" si="18"/>
-        <v>31.650000000000002</v>
-      </c>
-      <c r="AI14" s="7">
+        <v>0.6067170045961936</v>
+      </c>
+      <c r="AJ14" s="7">
         <f t="shared" si="19"/>
-        <v>0.6067170045961936</v>
-      </c>
-      <c r="AJ14" s="7">
+        <v>0.55653924981790326</v>
+      </c>
+      <c r="AK14" s="7">
         <f t="shared" si="20"/>
-        <v>0.55653924981790326</v>
-      </c>
-      <c r="AK14" s="7">
+        <v>0.73323891450854195</v>
+      </c>
+      <c r="AL14" s="7">
         <f t="shared" si="21"/>
-        <v>0.73323891450854195</v>
-      </c>
-      <c r="AL14" s="7">
-        <f t="shared" si="22"/>
         <v>0.69543899935770859</v>
       </c>
     </row>
@@ -2462,8 +2462,8 @@
         <v>9</v>
       </c>
       <c r="G15" s="4" t="str">
-        <f t="shared" si="12"/>
-        <v>TestAp_9</v>
+        <f t="shared" si="22"/>
+        <v>TestAp_09</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>82</v>
@@ -2520,46 +2520,46 @@
         <v>27931</v>
       </c>
       <c r="AA15" s="9">
+        <f t="shared" si="12"/>
+        <v>0.66150905617486688</v>
+      </c>
+      <c r="AB15" s="9">
         <f t="shared" si="13"/>
-        <v>0.66150905617486688</v>
-      </c>
-      <c r="AB15" s="9">
-        <f t="shared" si="14"/>
         <v>0.78332276343165064</v>
       </c>
       <c r="AD15" s="15" t="s">
         <v>41</v>
       </c>
       <c r="AE15" s="7">
+        <f t="shared" si="14"/>
+        <v>7.0953325150284838E-2</v>
+      </c>
+      <c r="AF15" s="7">
         <f t="shared" si="15"/>
-        <v>7.0953325150284838E-2</v>
-      </c>
-      <c r="AF15" s="7">
+        <v>5.1928500375294825E-2</v>
+      </c>
+      <c r="AG15" s="7">
         <f t="shared" si="16"/>
-        <v>5.1928500375294825E-2</v>
-      </c>
-      <c r="AG15" s="7">
+        <v>124.6</v>
+      </c>
+      <c r="AH15" s="7">
         <f t="shared" si="17"/>
-        <v>124.6</v>
-      </c>
-      <c r="AH15" s="7">
+        <v>42.075000000000003</v>
+      </c>
+      <c r="AI15" s="7">
         <f t="shared" si="18"/>
-        <v>42.075000000000003</v>
-      </c>
-      <c r="AI15" s="7">
+        <v>0.67019284381473787</v>
+      </c>
+      <c r="AJ15" s="7">
         <f t="shared" si="19"/>
-        <v>0.67019284381473787</v>
-      </c>
-      <c r="AJ15" s="7">
+        <v>0.62663440701875894</v>
+      </c>
+      <c r="AK15" s="7">
         <f t="shared" si="20"/>
-        <v>0.62663440701875894</v>
-      </c>
-      <c r="AK15" s="7">
+        <v>0.78945528360651618</v>
+      </c>
+      <c r="AL15" s="7">
         <f t="shared" si="21"/>
-        <v>0.78945528360651618</v>
-      </c>
-      <c r="AL15" s="7">
-        <f t="shared" si="22"/>
         <v>0.75869416835186942</v>
       </c>
     </row>
@@ -2584,7 +2584,7 @@
         <v>10</v>
       </c>
       <c r="G16" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_10</v>
       </c>
       <c r="H16" s="4" t="s">
@@ -2642,46 +2642,46 @@
         <v>27931</v>
       </c>
       <c r="AA16" s="9">
+        <f t="shared" si="12"/>
+        <v>0.60753473638187983</v>
+      </c>
+      <c r="AB16" s="9">
         <f t="shared" si="13"/>
-        <v>0.60753473638187983</v>
-      </c>
-      <c r="AB16" s="9">
-        <f t="shared" si="14"/>
         <v>0.73849415771205318</v>
       </c>
       <c r="AD16" s="15" t="s">
         <v>42</v>
       </c>
       <c r="AE16" s="7">
+        <f t="shared" si="14"/>
+        <v>8.3915382078617887E-2</v>
+      </c>
+      <c r="AF16" s="7">
         <f t="shared" si="15"/>
-        <v>8.3915382078617887E-2</v>
-      </c>
-      <c r="AF16" s="7">
+        <v>6.3615471182000102E-2</v>
+      </c>
+      <c r="AG16" s="7">
         <f t="shared" si="16"/>
-        <v>6.3615471182000102E-2</v>
-      </c>
-      <c r="AG16" s="7">
+        <v>129.69999999999999</v>
+      </c>
+      <c r="AH16" s="7">
         <f t="shared" si="17"/>
-        <v>129.69999999999999</v>
-      </c>
-      <c r="AH16" s="7">
+        <v>33.724999999999994</v>
+      </c>
+      <c r="AI16" s="7">
         <f t="shared" si="18"/>
-        <v>33.724999999999994</v>
-      </c>
-      <c r="AI16" s="7">
+        <v>0.61732785319911909</v>
+      </c>
+      <c r="AJ16" s="7">
         <f t="shared" si="19"/>
-        <v>0.61732785319911909</v>
-      </c>
-      <c r="AJ16" s="7">
+        <v>0.56820494996726423</v>
+      </c>
+      <c r="AK16" s="7">
         <f t="shared" si="20"/>
-        <v>0.56820494996726423</v>
-      </c>
-      <c r="AK16" s="7">
+        <v>0.74572820582022237</v>
+      </c>
+      <c r="AL16" s="7">
         <f t="shared" si="21"/>
-        <v>0.74572820582022237</v>
-      </c>
-      <c r="AL16" s="7">
-        <f t="shared" si="22"/>
         <v>0.70944175567121315</v>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
         <v>11</v>
       </c>
       <c r="G17" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_11</v>
       </c>
       <c r="H17" s="4" t="s">
@@ -2764,46 +2764,46 @@
         <v>27931</v>
       </c>
       <c r="AA17" s="9">
+        <f t="shared" si="12"/>
+        <v>0.74337969529372117</v>
+      </c>
+      <c r="AB17" s="9">
         <f t="shared" si="13"/>
-        <v>0.74337969529372117</v>
-      </c>
-      <c r="AB17" s="9">
-        <f t="shared" si="14"/>
         <v>0.83103487495676698</v>
       </c>
       <c r="AD17" s="15" t="s">
         <v>98</v>
       </c>
       <c r="AE17" s="7">
+        <f t="shared" si="14"/>
+        <v>5.2314399581055604E-2</v>
+      </c>
+      <c r="AF17" s="7">
         <f t="shared" si="15"/>
-        <v>5.2314399581055604E-2</v>
-      </c>
-      <c r="AF17" s="7">
+        <v>3.9884330119963021E-2</v>
+      </c>
+      <c r="AG17" s="7">
         <f t="shared" si="16"/>
-        <v>3.9884330119963021E-2</v>
-      </c>
-      <c r="AG17" s="7">
+        <v>220.75</v>
+      </c>
+      <c r="AH17" s="7">
         <f t="shared" si="17"/>
-        <v>220.75</v>
-      </c>
-      <c r="AH17" s="7">
+        <v>53.405000000000001</v>
+      </c>
+      <c r="AI17" s="7">
         <f t="shared" si="18"/>
-        <v>53.405000000000001</v>
-      </c>
-      <c r="AI17" s="7">
+        <v>0.75020997772912867</v>
+      </c>
+      <c r="AJ17" s="7">
         <f t="shared" si="19"/>
-        <v>0.75020997772912867</v>
-      </c>
-      <c r="AJ17" s="7">
+        <v>0.71594884213947385</v>
+      </c>
+      <c r="AK17" s="7">
         <f t="shared" si="20"/>
-        <v>0.71594884213947385</v>
-      </c>
-      <c r="AK17" s="7">
+        <v>0.83592507534542093</v>
+      </c>
+      <c r="AL17" s="7">
         <f t="shared" si="21"/>
-        <v>0.83592507534542093</v>
-      </c>
-      <c r="AL17" s="7">
-        <f t="shared" si="22"/>
         <v>0.81139551596618864</v>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
         <v>12</v>
       </c>
       <c r="G18" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_12</v>
       </c>
       <c r="H18" s="4" t="s">
@@ -2886,46 +2886,46 @@
         <v>27931</v>
       </c>
       <c r="AA18" s="9">
+        <f t="shared" si="12"/>
+        <v>0.75174047215563766</v>
+      </c>
+      <c r="AB18" s="9">
         <f t="shared" si="13"/>
-        <v>0.75174047215563766</v>
-      </c>
-      <c r="AB18" s="9">
-        <f t="shared" si="14"/>
         <v>0.83882434038122455</v>
       </c>
       <c r="AD18" s="15" t="s">
         <v>21</v>
       </c>
       <c r="AE18" s="7">
+        <f t="shared" si="14"/>
+        <v>5.0473020999693675E-2</v>
+      </c>
+      <c r="AF18" s="7">
         <f t="shared" si="15"/>
-        <v>5.0473020999693675E-2</v>
-      </c>
-      <c r="AF18" s="7">
+        <v>3.7954056186406002E-2</v>
+      </c>
+      <c r="AG18" s="7">
         <f t="shared" si="16"/>
-        <v>3.7954056186406002E-2</v>
-      </c>
-      <c r="AG18" s="7">
+        <v>208.2</v>
+      </c>
+      <c r="AH18" s="7">
         <f t="shared" si="17"/>
-        <v>208.2</v>
-      </c>
-      <c r="AH18" s="7">
+        <v>56.524999999999999</v>
+      </c>
+      <c r="AI18" s="7">
         <f t="shared" si="18"/>
-        <v>56.524999999999999</v>
-      </c>
-      <c r="AI18" s="7">
+        <v>0.75837110278516462</v>
+      </c>
+      <c r="AJ18" s="7">
         <f t="shared" si="19"/>
-        <v>0.75837110278516462</v>
-      </c>
-      <c r="AJ18" s="7">
+        <v>0.72511143348283857</v>
+      </c>
+      <c r="AK18" s="7">
         <f t="shared" si="20"/>
-        <v>0.72511143348283857</v>
-      </c>
-      <c r="AK18" s="7">
+        <v>0.84350532891111429</v>
+      </c>
+      <c r="AL18" s="7">
         <f t="shared" si="21"/>
-        <v>0.84350532891111429</v>
-      </c>
-      <c r="AL18" s="7">
-        <f t="shared" si="22"/>
         <v>0.8200251896587758</v>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
         <v>13</v>
       </c>
       <c r="G19" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_13</v>
       </c>
       <c r="H19" s="4" t="s">
@@ -3008,46 +3008,46 @@
         <v>27931</v>
       </c>
       <c r="AA19" s="9">
+        <f t="shared" si="12"/>
+        <v>0.76559357812699225</v>
+      </c>
+      <c r="AB19" s="9">
         <f t="shared" si="13"/>
-        <v>0.76559357812699225</v>
-      </c>
-      <c r="AB19" s="9">
-        <f t="shared" si="14"/>
         <v>0.85247668983121827</v>
       </c>
       <c r="AD19" s="15" t="s">
         <v>20</v>
       </c>
       <c r="AE19" s="7">
+        <f t="shared" si="14"/>
+        <v>4.7445478974433256E-2</v>
+      </c>
+      <c r="AF19" s="7">
         <f t="shared" si="15"/>
-        <v>4.7445478974433256E-2</v>
-      </c>
-      <c r="AF19" s="7">
+        <v>3.4594246662871191E-2</v>
+      </c>
+      <c r="AG19" s="7">
         <f t="shared" si="16"/>
-        <v>3.4594246662871191E-2</v>
-      </c>
-      <c r="AG19" s="7">
+        <v>185.05</v>
+      </c>
+      <c r="AH19" s="7">
         <f t="shared" si="17"/>
-        <v>185.05</v>
-      </c>
-      <c r="AH19" s="7">
+        <v>63.05</v>
+      </c>
+      <c r="AI19" s="7">
         <f t="shared" si="18"/>
-        <v>63.05</v>
-      </c>
-      <c r="AI19" s="7">
+        <v>0.77188948175717731</v>
+      </c>
+      <c r="AJ19" s="7">
         <f t="shared" si="19"/>
-        <v>0.77188948175717731</v>
-      </c>
-      <c r="AJ19" s="7">
+        <v>0.74030882459211311</v>
+      </c>
+      <c r="AK19" s="7">
         <f t="shared" si="20"/>
-        <v>0.74030882459211311</v>
-      </c>
-      <c r="AK19" s="7">
+        <v>0.85678686544170934</v>
+      </c>
+      <c r="AL19" s="7">
         <f t="shared" si="21"/>
-        <v>0.85678686544170934</v>
-      </c>
-      <c r="AL19" s="7">
-        <f t="shared" si="22"/>
         <v>0.83516674762041077</v>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
         <v>14</v>
       </c>
       <c r="G20" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_14</v>
       </c>
       <c r="H20" s="4" t="s">
@@ -3130,46 +3130,46 @@
         <v>27931</v>
       </c>
       <c r="AA20" s="9">
+        <f t="shared" si="12"/>
+        <v>0.79959172215838858</v>
+      </c>
+      <c r="AB20" s="9">
         <f t="shared" si="13"/>
-        <v>0.79959172215838858</v>
-      </c>
-      <c r="AB20" s="9">
-        <f t="shared" si="14"/>
         <v>0.87503430175298669</v>
       </c>
       <c r="AD20" s="15" t="s">
         <v>22</v>
       </c>
       <c r="AE20" s="7">
+        <f t="shared" si="14"/>
+        <v>4.0134718945301948E-2</v>
+      </c>
+      <c r="AF20" s="7">
         <f t="shared" si="15"/>
-        <v>4.0134718945301948E-2</v>
-      </c>
-      <c r="AF20" s="7">
+        <v>2.9106147111298133E-2</v>
+      </c>
+      <c r="AG20" s="7">
         <f t="shared" si="16"/>
-        <v>2.9106147111298133E-2</v>
-      </c>
-      <c r="AG20" s="7">
+        <v>213.55</v>
+      </c>
+      <c r="AH20" s="7">
         <f t="shared" si="17"/>
-        <v>213.55</v>
-      </c>
-      <c r="AH20" s="7">
+        <v>75.075000000000003</v>
+      </c>
+      <c r="AI20" s="7">
         <f t="shared" si="18"/>
-        <v>75.075000000000003</v>
-      </c>
-      <c r="AI20" s="7">
+        <v>0.80504619437471781</v>
+      </c>
+      <c r="AJ20" s="7">
         <f t="shared" si="19"/>
-        <v>0.80504619437471781</v>
-      </c>
-      <c r="AJ20" s="7">
+        <v>0.77768621124943571</v>
+      </c>
+      <c r="AK20" s="7">
         <f t="shared" si="20"/>
-        <v>0.77768621124943571</v>
-      </c>
-      <c r="AK20" s="7">
+        <v>0.87872057152465455</v>
+      </c>
+      <c r="AL20" s="7">
         <f t="shared" si="21"/>
-        <v>0.87872057152465455</v>
-      </c>
-      <c r="AL20" s="7">
-        <f t="shared" si="22"/>
         <v>0.86023000548122819</v>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
         <v>15</v>
       </c>
       <c r="G21" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_15</v>
       </c>
       <c r="H21" s="4" t="s">
@@ -3252,46 +3252,46 @@
         <v>27931</v>
       </c>
       <c r="AA21" s="9">
+        <f t="shared" si="12"/>
+        <v>0.75982305247542281</v>
+      </c>
+      <c r="AB21" s="9">
         <f t="shared" si="13"/>
-        <v>0.75982305247542281</v>
-      </c>
-      <c r="AB21" s="9">
-        <f t="shared" si="14"/>
         <v>0.8466477160452357</v>
       </c>
       <c r="AD21" s="15" t="s">
         <v>23</v>
       </c>
       <c r="AE21" s="7">
+        <f t="shared" si="14"/>
+        <v>4.8703088335889717E-2</v>
+      </c>
+      <c r="AF21" s="7">
         <f t="shared" si="15"/>
-        <v>4.8703088335889717E-2</v>
-      </c>
-      <c r="AF21" s="7">
+        <v>3.6025146253839117E-2</v>
+      </c>
+      <c r="AG21" s="7">
         <f t="shared" si="16"/>
-        <v>3.6025146253839117E-2</v>
-      </c>
-      <c r="AG21" s="7">
+        <v>195.10000000000002</v>
+      </c>
+      <c r="AH21" s="7">
         <f t="shared" si="17"/>
-        <v>195.10000000000002</v>
-      </c>
-      <c r="AH21" s="7">
+        <v>60.075000000000003</v>
+      </c>
+      <c r="AI21" s="7">
         <f t="shared" si="18"/>
-        <v>60.075000000000003</v>
-      </c>
-      <c r="AI21" s="7">
+        <v>0.76625897446023483</v>
+      </c>
+      <c r="AJ21" s="7">
         <f t="shared" si="19"/>
-        <v>0.76625897446023483</v>
-      </c>
-      <c r="AJ21" s="7">
+        <v>0.73397597623119748</v>
+      </c>
+      <c r="AK21" s="7">
         <f t="shared" si="20"/>
-        <v>0.73397597623119748</v>
-      </c>
-      <c r="AK21" s="7">
+        <v>0.85111685056599706</v>
+      </c>
+      <c r="AL21" s="7">
         <f t="shared" si="21"/>
-        <v>0.85111685056599706</v>
-      </c>
-      <c r="AL21" s="7">
-        <f t="shared" si="22"/>
         <v>0.82869938463655579</v>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
         <v>16</v>
       </c>
       <c r="G22" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_16</v>
       </c>
       <c r="H22" s="4" t="s">
@@ -3374,46 +3374,46 @@
         <v>27931</v>
       </c>
       <c r="AA22" s="9">
+        <f t="shared" si="12"/>
+        <v>0.6878707301214726</v>
+      </c>
+      <c r="AB22" s="9">
         <f t="shared" si="13"/>
-        <v>0.6878707301214726</v>
-      </c>
-      <c r="AB22" s="9">
-        <f t="shared" si="14"/>
         <v>0.79641121239988555</v>
       </c>
       <c r="AD22" s="15" t="s">
         <v>26</v>
       </c>
       <c r="AE22" s="7">
+        <f t="shared" si="14"/>
+        <v>6.4825577175264812E-2</v>
+      </c>
+      <c r="AF22" s="7">
         <f t="shared" si="15"/>
-        <v>6.4825577175264812E-2</v>
-      </c>
-      <c r="AF22" s="7">
+        <v>4.8585650198014883E-2</v>
+      </c>
+      <c r="AG22" s="7">
         <f t="shared" si="16"/>
-        <v>4.8585650198014883E-2</v>
-      </c>
-      <c r="AG22" s="7">
+        <v>157.35000000000002</v>
+      </c>
+      <c r="AH22" s="7">
         <f t="shared" si="17"/>
-        <v>157.35000000000002</v>
-      </c>
-      <c r="AH22" s="7">
+        <v>44.325000000000003</v>
+      </c>
+      <c r="AI22" s="7">
         <f t="shared" si="18"/>
-        <v>44.325000000000003</v>
-      </c>
-      <c r="AI22" s="7">
+        <v>0.69597878263785262</v>
+      </c>
+      <c r="AJ22" s="7">
         <f t="shared" si="19"/>
-        <v>0.69597878263785262</v>
-      </c>
-      <c r="AJ22" s="7">
+        <v>0.65530827021633242</v>
+      </c>
+      <c r="AK22" s="7">
         <f t="shared" si="20"/>
-        <v>0.65530827021633242</v>
-      </c>
-      <c r="AK22" s="7">
+        <v>0.80220982943996211</v>
+      </c>
+      <c r="AL22" s="7">
         <f t="shared" si="21"/>
-        <v>0.80220982943996211</v>
-      </c>
-      <c r="AL22" s="7">
-        <f t="shared" si="22"/>
         <v>0.77312359376503981</v>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
         <v>17</v>
       </c>
       <c r="G23" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_17</v>
       </c>
       <c r="H23" s="4" t="s">
@@ -3496,46 +3496,46 @@
         <v>27931</v>
       </c>
       <c r="AA23" s="9">
+        <f t="shared" si="12"/>
+        <v>0.83921407971329132</v>
+      </c>
+      <c r="AB23" s="9">
         <f t="shared" si="13"/>
-        <v>0.83921407971329132</v>
-      </c>
-      <c r="AB23" s="9">
-        <f t="shared" si="14"/>
         <v>0.90499959760490523</v>
       </c>
       <c r="AD23" s="15" t="s">
         <v>80</v>
       </c>
       <c r="AE23" s="7">
+        <f t="shared" si="14"/>
+        <v>3.1816635563952117E-2</v>
+      </c>
+      <c r="AF23" s="7">
         <f t="shared" si="15"/>
-        <v>3.1816635563952117E-2</v>
-      </c>
-      <c r="AF23" s="7">
+        <v>2.193281203171403E-2</v>
+      </c>
+      <c r="AG23" s="7">
         <f t="shared" si="16"/>
-        <v>2.193281203171403E-2</v>
-      </c>
-      <c r="AG23" s="7">
+        <v>215.89999999999998</v>
+      </c>
+      <c r="AH23" s="7">
         <f t="shared" si="17"/>
-        <v>215.89999999999998</v>
-      </c>
-      <c r="AH23" s="7">
+        <v>102.425</v>
+      </c>
+      <c r="AI23" s="7">
         <f t="shared" si="18"/>
-        <v>102.425</v>
-      </c>
-      <c r="AI23" s="7">
+        <v>0.84365416500448298</v>
+      </c>
+      <c r="AJ23" s="7">
         <f t="shared" si="19"/>
-        <v>0.84365416500448298</v>
-      </c>
-      <c r="AJ23" s="7">
+        <v>0.82138241187718053</v>
+      </c>
+      <c r="AK23" s="7">
         <f t="shared" si="20"/>
-        <v>0.82138241187718053</v>
-      </c>
-      <c r="AK23" s="7">
+        <v>0.90783633750191561</v>
+      </c>
+      <c r="AL23" s="7">
         <f t="shared" si="21"/>
-        <v>0.90783633750191561</v>
-      </c>
-      <c r="AL23" s="7">
-        <f t="shared" si="22"/>
         <v>0.89360706789803568</v>
       </c>
     </row>
@@ -3560,7 +3560,7 @@
         <v>18</v>
       </c>
       <c r="G24" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_18</v>
       </c>
       <c r="H24" s="4" t="s">
@@ -3618,46 +3618,46 @@
         <v>27931</v>
       </c>
       <c r="AA24" s="9">
+        <f t="shared" si="12"/>
+        <v>0.80572125872845124</v>
+      </c>
+      <c r="AB24" s="9">
         <f t="shared" si="13"/>
-        <v>0.80572125872845124</v>
-      </c>
-      <c r="AB24" s="9">
-        <f t="shared" si="14"/>
         <v>0.87393282945805528</v>
       </c>
       <c r="AD24" s="15" t="s">
         <v>25</v>
       </c>
       <c r="AE24" s="7">
+        <f t="shared" si="14"/>
+        <v>3.8834069482727399E-2</v>
+      </c>
+      <c r="AF24" s="7">
         <f t="shared" si="15"/>
-        <v>3.8834069482727399E-2</v>
-      </c>
-      <c r="AF24" s="7">
+        <v>2.9372336546430823E-2</v>
+      </c>
+      <c r="AG24" s="7">
         <f t="shared" si="16"/>
-        <v>2.9372336546430823E-2</v>
-      </c>
-      <c r="AG24" s="7">
+        <v>283.3</v>
+      </c>
+      <c r="AH24" s="7">
         <f t="shared" si="17"/>
-        <v>283.3</v>
-      </c>
-      <c r="AH24" s="7">
+        <v>72.7</v>
+      </c>
+      <c r="AI24" s="7">
         <f t="shared" si="18"/>
-        <v>72.7</v>
-      </c>
-      <c r="AI24" s="7">
+        <v>0.81102112038168983</v>
+      </c>
+      <c r="AJ24" s="7">
         <f t="shared" si="19"/>
-        <v>0.81102112038168983</v>
-      </c>
-      <c r="AJ24" s="7">
+        <v>0.78443667377568604</v>
+      </c>
+      <c r="AK24" s="7">
         <f t="shared" si="20"/>
-        <v>0.78443667377568604</v>
-      </c>
-      <c r="AK24" s="7">
+        <v>0.87764988152353141</v>
+      </c>
+      <c r="AL24" s="7">
         <f t="shared" si="21"/>
-        <v>0.87764988152353141</v>
-      </c>
-      <c r="AL24" s="7">
-        <f t="shared" si="22"/>
         <v>0.8590049095163842</v>
       </c>
     </row>
@@ -3682,7 +3682,7 @@
         <v>19</v>
       </c>
       <c r="G25" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_19</v>
       </c>
       <c r="H25" s="4" t="s">
@@ -3740,46 +3740,46 @@
         <v>27931</v>
       </c>
       <c r="AA25" s="9">
+        <f t="shared" si="12"/>
+        <v>0.81136917550751486</v>
+      </c>
+      <c r="AB25" s="9">
         <f t="shared" si="13"/>
-        <v>0.81136917550751486</v>
-      </c>
-      <c r="AB25" s="9">
-        <f t="shared" si="14"/>
         <v>0.88449912490103977</v>
       </c>
       <c r="AD25" s="15" t="s">
         <v>29</v>
       </c>
       <c r="AE25" s="7">
+        <f t="shared" si="14"/>
+        <v>3.7640184864424775E-2</v>
+      </c>
+      <c r="AF25" s="7">
         <f t="shared" si="15"/>
-        <v>3.7640184864424775E-2</v>
-      </c>
-      <c r="AF25" s="7">
+        <v>2.6826240066875125E-2</v>
+      </c>
+      <c r="AG25" s="7">
         <f t="shared" si="16"/>
-        <v>2.6826240066875125E-2</v>
-      </c>
-      <c r="AG25" s="7">
+        <v>209.5</v>
+      </c>
+      <c r="AH25" s="7">
         <f t="shared" si="17"/>
-        <v>209.5</v>
-      </c>
-      <c r="AH25" s="7">
+        <v>82.224999999999994</v>
+      </c>
+      <c r="AI25" s="7">
         <f t="shared" si="18"/>
-        <v>82.224999999999994</v>
-      </c>
-      <c r="AI25" s="7">
+        <v>0.81652581172340544</v>
+      </c>
+      <c r="AJ25" s="7">
         <f t="shared" si="19"/>
-        <v>0.81652581172340544</v>
-      </c>
-      <c r="AJ25" s="7">
+        <v>0.79065979311438017</v>
+      </c>
+      <c r="AK25" s="7">
         <f t="shared" si="20"/>
-        <v>0.79065979311438017</v>
-      </c>
-      <c r="AK25" s="7">
+        <v>0.88791956931990623</v>
+      </c>
+      <c r="AL25" s="7">
         <f t="shared" si="21"/>
-        <v>0.88791956931990623</v>
-      </c>
-      <c r="AL25" s="7">
-        <f t="shared" si="22"/>
         <v>0.87076240032727859</v>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
         <v>20</v>
       </c>
       <c r="G26" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_20</v>
       </c>
       <c r="H26" s="4" t="s">
@@ -3862,46 +3862,46 @@
         <v>27931</v>
       </c>
       <c r="AA26" s="9">
+        <f t="shared" si="12"/>
+        <v>0.8300100459967491</v>
+      </c>
+      <c r="AB26" s="9">
         <f t="shared" si="13"/>
-        <v>0.8300100459967491</v>
-      </c>
-      <c r="AB26" s="9">
-        <f t="shared" si="14"/>
         <v>0.89924012202056558</v>
       </c>
       <c r="AD26" s="15" t="s">
         <v>74</v>
       </c>
       <c r="AE26" s="7">
+        <f t="shared" si="14"/>
+        <v>3.37302774349496E-2</v>
+      </c>
+      <c r="AF26" s="7">
         <f t="shared" si="15"/>
-        <v>3.37302774349496E-2</v>
-      </c>
-      <c r="AF26" s="7">
+        <v>2.3301491904001419E-2</v>
+      </c>
+      <c r="AG26" s="7">
         <f t="shared" si="16"/>
-        <v>2.3301491904001419E-2</v>
-      </c>
-      <c r="AG26" s="7">
+        <v>205.14999999999998</v>
+      </c>
+      <c r="AH26" s="7">
         <f t="shared" si="17"/>
-        <v>205.14999999999998</v>
-      </c>
-      <c r="AH26" s="7">
+        <v>96.325000000000003</v>
+      </c>
+      <c r="AI26" s="7">
         <f t="shared" si="18"/>
-        <v>96.325000000000003</v>
-      </c>
-      <c r="AI26" s="7">
+        <v>0.83468887443025308</v>
+      </c>
+      <c r="AJ26" s="7">
         <f t="shared" si="19"/>
-        <v>0.83468887443025308</v>
-      </c>
-      <c r="AJ26" s="7">
+        <v>0.81121957036018699</v>
+      </c>
+      <c r="AK26" s="7">
         <f t="shared" si="20"/>
-        <v>0.81121957036018699</v>
-      </c>
-      <c r="AK26" s="7">
+        <v>0.90224193075651904</v>
+      </c>
+      <c r="AL26" s="7">
         <f t="shared" si="21"/>
-        <v>0.90224193075651904</v>
-      </c>
-      <c r="AL26" s="7">
-        <f t="shared" si="22"/>
         <v>0.88718466524966821</v>
       </c>
     </row>
@@ -3926,7 +3926,7 @@
         <v>21</v>
       </c>
       <c r="G27" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_21</v>
       </c>
       <c r="H27" s="4" t="s">
@@ -3984,43 +3984,43 @@
         <v>27931</v>
       </c>
       <c r="AA27" s="9">
+        <f t="shared" si="12"/>
+        <v>0.73431094886686066</v>
+      </c>
+      <c r="AB27" s="9">
         <f t="shared" si="13"/>
-        <v>0.73431094886686066</v>
-      </c>
-      <c r="AB27" s="9">
+        <v>0.83143743150974181</v>
+      </c>
+      <c r="AE27" s="7">
         <f t="shared" si="14"/>
-        <v>0.83143743150974181</v>
-      </c>
-      <c r="AE27" s="7">
+        <v>5.4324022253522293E-2</v>
+      </c>
+      <c r="AF27" s="7">
         <f t="shared" si="15"/>
-        <v>5.4324022253522293E-2</v>
-      </c>
-      <c r="AF27" s="7">
+        <v>3.9784334174003483E-2</v>
+      </c>
+      <c r="AG27" s="7">
         <f t="shared" si="16"/>
-        <v>3.9784334174003483E-2</v>
-      </c>
-      <c r="AG27" s="7">
+        <v>164.85</v>
+      </c>
+      <c r="AH27" s="7">
         <f t="shared" si="17"/>
-        <v>164.85</v>
-      </c>
-      <c r="AH27" s="7">
+        <v>54.75</v>
+      </c>
+      <c r="AI27" s="7">
         <f t="shared" si="18"/>
-        <v>54.75</v>
-      </c>
-      <c r="AI27" s="7">
+        <v>0.74135573072334071</v>
+      </c>
+      <c r="AJ27" s="7">
         <f t="shared" si="19"/>
-        <v>0.74135573072334071</v>
-      </c>
-      <c r="AJ27" s="7">
+        <v>0.70601865225449123</v>
+      </c>
+      <c r="AK27" s="7">
         <f t="shared" si="20"/>
-        <v>0.70601865225449123</v>
-      </c>
-      <c r="AK27" s="7">
+        <v>0.83631686247873549</v>
+      </c>
+      <c r="AL27" s="7">
         <f t="shared" si="21"/>
-        <v>0.83631686247873549</v>
-      </c>
-      <c r="AL27" s="7">
-        <f t="shared" si="22"/>
         <v>0.81184132320053026</v>
       </c>
     </row>
@@ -4045,7 +4045,7 @@
         <v>22</v>
       </c>
       <c r="G28" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_22</v>
       </c>
       <c r="H28" s="4" t="s">
@@ -4103,11 +4103,11 @@
         <v>27931</v>
       </c>
       <c r="AA28" s="9">
+        <f t="shared" si="12"/>
+        <v>0.77006864595145863</v>
+      </c>
+      <c r="AB28" s="9">
         <f t="shared" si="13"/>
-        <v>0.77006864595145863</v>
-      </c>
-      <c r="AB28" s="9">
-        <f t="shared" si="14"/>
         <v>0.85335198674119073</v>
       </c>
       <c r="AE28" s="7">
@@ -4164,7 +4164,7 @@
         <v>23</v>
       </c>
       <c r="G29" s="4" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="22"/>
         <v>TestAp_23</v>
       </c>
       <c r="H29" s="4" t="s">
@@ -4222,11 +4222,11 @@
         <v>27931</v>
       </c>
       <c r="AA29" s="9">
+        <f t="shared" si="12"/>
+        <v>0.69069609834421586</v>
+      </c>
+      <c r="AB29" s="9">
         <f t="shared" si="13"/>
-        <v>0.69069609834421586</v>
-      </c>
-      <c r="AB29" s="9">
-        <f t="shared" si="14"/>
         <v>0.80015125722736158</v>
       </c>
       <c r="AE29" s="7">
@@ -4283,7 +4283,7 @@
         <v>24</v>
       </c>
       <c r="G30" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="22"/>
         <v>TestAp_24</v>
       </c>
       <c r="H30" s="4" t="s">
@@ -4402,7 +4402,7 @@
         <v>25</v>
       </c>
       <c r="G31" s="4" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="22"/>
         <v>TestAp_25</v>
       </c>
       <c r="H31" s="4" t="s">
@@ -4521,8 +4521,8 @@
         <v>1</v>
       </c>
       <c r="G32" s="4" t="str">
-        <f t="shared" si="4"/>
-        <v>TestZir_1</v>
+        <f t="shared" si="22"/>
+        <v>TestZir_01</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>83</v>
@@ -4640,8 +4640,8 @@
         <v>2</v>
       </c>
       <c r="G33" s="4" t="str">
-        <f t="shared" si="4"/>
-        <v>TestZir_2</v>
+        <f t="shared" si="22"/>
+        <v>TestZir_02</v>
       </c>
       <c r="H33" s="4" t="s">
         <v>83</v>
@@ -4759,8 +4759,8 @@
         <v>3</v>
       </c>
       <c r="G34" s="4" t="str">
-        <f t="shared" si="4"/>
-        <v>TestZir_3</v>
+        <f t="shared" si="22"/>
+        <v>TestZir_03</v>
       </c>
       <c r="H34" s="4" t="s">
         <v>83</v>
@@ -4878,8 +4878,8 @@
         <v>4</v>
       </c>
       <c r="G35" s="4" t="str">
-        <f t="shared" si="4"/>
-        <v>TestZir_4</v>
+        <f t="shared" si="22"/>
+        <v>TestZir_04</v>
       </c>
       <c r="H35" s="4" t="s">
         <v>83</v>
@@ -4997,8 +4997,8 @@
         <v>5</v>
       </c>
       <c r="G36" s="4" t="str">
-        <f t="shared" si="4"/>
-        <v>TestZir_5</v>
+        <f t="shared" si="22"/>
+        <v>TestZir_05</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>83</v>
@@ -5116,8 +5116,8 @@
         <v>6</v>
       </c>
       <c r="G37" s="4" t="str">
-        <f t="shared" si="4"/>
-        <v>TestZir_6</v>
+        <f t="shared" si="22"/>
+        <v>TestZir_06</v>
       </c>
       <c r="H37" s="4" t="s">
         <v>83</v>

</xml_diff>